<commit_message>
refactor: departemen to divisi in karyawan
</commit_message>
<xml_diff>
--- a/public/assets/static/template/template-import-karyawan.xlsx
+++ b/public/assets/static/template/template-import-karyawan.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\akmal\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Program\Laravel\Profile karyawan\public\assets\static\template\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B15E44B2-5F13-47EF-A623-37CC605C3087}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B0C9047C-ECBF-4F36-9A46-E023ECD4659A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
   <si>
     <t>nip</t>
   </si>
@@ -34,9 +34,6 @@
     <t>email</t>
   </si>
   <si>
-    <t>jabatan</t>
-  </si>
-  <si>
     <t>no_hp</t>
   </si>
   <si>
@@ -52,20 +49,20 @@
     <t>alamat</t>
   </si>
   <si>
-    <t>status</t>
-  </si>
-  <si>
     <t>divisi</t>
   </si>
   <si>
     <t>departemen</t>
+  </si>
+  <si>
+    <t>posisi</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
+  <fonts count="3">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -79,6 +76,13 @@
       <color theme="10"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -99,20 +103,235 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="2">
+  <cellStyles count="3">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal 2" xfId="2" xr:uid="{2F83BFF7-ED8F-4D52-85E5-A96D235B897A}"/>
   </cellStyles>
-  <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <dxfs count="17">
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4" tint="0.79995117038483843"/>
+          <bgColor theme="4" tint="0.79995117038483843"/>
+        </patternFill>
+      </fill>
+      <border>
+        <bottom style="thin">
+          <color theme="4" tint="0.39994506668294322"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4" tint="0.79995117038483843"/>
+          <bgColor theme="4" tint="0.79995117038483843"/>
+        </patternFill>
+      </fill>
+      <border>
+        <bottom style="thin">
+          <color theme="4" tint="0.39994506668294322"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+      <border>
+        <bottom style="thin">
+          <color theme="4" tint="0.39994506668294322"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color theme="1"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color theme="1"/>
+      </font>
+      <border>
+        <top style="thin">
+          <color theme="4"/>
+        </top>
+        <bottom style="thin">
+          <color theme="4"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4" tint="0.79995117038483843"/>
+          <bgColor theme="4" tint="0.79995117038483843"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4" tint="0.79995117038483843"/>
+          <bgColor theme="4" tint="0.79995117038483843"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color theme="1"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4" tint="0.79995117038483843"/>
+          <bgColor theme="4" tint="0.79995117038483843"/>
+        </patternFill>
+      </fill>
+      <border>
+        <top style="thin">
+          <color theme="4" tint="0.39994506668294322"/>
+        </top>
+        <bottom style="thin">
+          <color theme="4" tint="0.39994506668294322"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color theme="1"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4" tint="0.79995117038483843"/>
+          <bgColor theme="4" tint="0.79995117038483843"/>
+        </patternFill>
+      </fill>
+      <border>
+        <bottom style="thin">
+          <color theme="4" tint="0.39994506668294322"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4" tint="0.79995117038483843"/>
+          <bgColor theme="4" tint="0.79995117038483843"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4" tint="0.79995117038483843"/>
+          <bgColor theme="4" tint="0.79995117038483843"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color theme="1"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color theme="1"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color theme="1"/>
+      </font>
+      <border>
+        <top style="double">
+          <color theme="4"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4"/>
+          <bgColor theme="4"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+      <border>
+        <left style="thin">
+          <color theme="4"/>
+        </left>
+        <right style="thin">
+          <color theme="4"/>
+        </right>
+        <top style="thin">
+          <color theme="4"/>
+        </top>
+        <bottom style="thin">
+          <color theme="4"/>
+        </bottom>
+        <horizontal style="thin">
+          <color theme="4" tint="0.39994506668294322"/>
+        </horizontal>
+      </border>
+    </dxf>
+  </dxfs>
+  <tableStyles count="2" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16">
+    <tableStyle name="TableStylePreset3_Accent1" pivot="0" count="7" xr9:uid="{1CB9243F-18E8-40BA-B8C5-0EEE534D86A2}">
+      <tableStyleElement type="wholeTable" dxfId="16"/>
+      <tableStyleElement type="headerRow" dxfId="15"/>
+      <tableStyleElement type="totalRow" dxfId="14"/>
+      <tableStyleElement type="firstColumn" dxfId="13"/>
+      <tableStyleElement type="lastColumn" dxfId="12"/>
+      <tableStyleElement type="firstRowStripe" dxfId="11"/>
+      <tableStyleElement type="firstColumnStripe" dxfId="10"/>
+    </tableStyle>
+    <tableStyle name="PivotStylePreset2_Accent1" table="0" count="10" xr9:uid="{86CB95D6-921F-4213-9CA4-8E2987812321}">
+      <tableStyleElement type="headerRow" dxfId="9"/>
+      <tableStyleElement type="totalRow" dxfId="8"/>
+      <tableStyleElement type="firstRowStripe" dxfId="7"/>
+      <tableStyleElement type="firstColumnStripe" dxfId="6"/>
+      <tableStyleElement type="firstSubtotalRow" dxfId="5"/>
+      <tableStyleElement type="secondSubtotalRow" dxfId="4"/>
+      <tableStyleElement type="firstRowSubheading" dxfId="3"/>
+      <tableStyleElement type="secondRowSubheading" dxfId="2"/>
+      <tableStyleElement type="pageFieldLabels" dxfId="1"/>
+      <tableStyleElement type="pageFieldValues" dxfId="0"/>
+    </tableStyle>
+  </tableStyles>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -409,25 +628,24 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:M2"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:L2"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="5.81640625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="11.81640625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="14.08984375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="24.453125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.90625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="10.08984375" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="13.36328125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="5.81640625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="10.90625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="12.36328125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.90625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.36328125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="24.453125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="12.90625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="10.08984375" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="13.36328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:12">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -438,38 +656,35 @@
         <v>2</v>
       </c>
       <c r="D1" t="s">
+        <v>9</v>
+      </c>
+      <c r="E1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="G1" t="s">
+        <v>11</v>
+      </c>
+      <c r="H1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="I1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="J1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="K1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="L1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
-        <v>9</v>
-      </c>
-      <c r="K1" t="s">
-        <v>10</v>
-      </c>
-      <c r="L1" t="s">
-        <v>11</v>
-      </c>
-      <c r="M1" t="s">
-        <v>12</v>
-      </c>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="D2" s="1"/>
+    <row r="2" spans="1:12">
+      <c r="F2" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>